<commit_message>
Added profile examples to manually loaded metadata. Fixed issues with transient profile event functions not being called with the correct data.
</commit_message>
<xml_diff>
--- a/src/rattlesnake/examples/environment/random/random_v3.xlsx
+++ b/src/rattlesnake/examples/environment/random/random_v3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\examples\environment\random\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\rattlesnake-vibration-controller-headless\src\rattlesnake\examples\environment\random\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{370CE37A-8FB1-4197-8881-D6B66A185A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21278725-BF82-47ED-907C-33670AF2E744}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6070" yWindow="1960" windowWidth="28790" windowHeight="15350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Random 0" sheetId="3" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="51">
   <si>
     <t>Random 0</t>
   </si>
@@ -171,6 +171,9 @@
   </si>
   <si>
     <t>Disarm DAQ</t>
+  </si>
+  <si>
+    <t>Save Control Data</t>
   </si>
 </sst>
 </file>
@@ -1053,7 +1056,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="18.08984375" bestFit="1" customWidth="1"/>
@@ -1092,75 +1095,97 @@
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
         <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>44</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
         <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
         <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>40</v>
+      </c>
+      <c r="B10" t="s">
         <v>42</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>40</v>
+      </c>
+      <c r="B11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" t="s">
         <v>49</v>
       </c>
     </row>

</xml_diff>